<commit_message>
docs: update product vision PDF and assets
</commit_message>
<xml_diff>
--- a/backend/data/Project_NourishBot.xlsx
+++ b/backend/data/Project_NourishBot.xlsx
@@ -18262,7 +18262,7 @@
       </c>
       <c r="F2" s="16" t="inlineStr">
         <is>
-          <t>rajesh.kumar@dzukku.com</t>
+          <t>rajesh.kumar@nourishbot.local</t>
         </is>
       </c>
       <c r="G2" s="16" t="inlineStr">
@@ -18329,7 +18329,7 @@
       </c>
       <c r="F3" s="16" t="inlineStr">
         <is>
-          <t>priya.sharma@dzukku.com</t>
+          <t>priya.sharma@nourishbot.local</t>
         </is>
       </c>
       <c r="G3" s="16" t="inlineStr">
@@ -18396,7 +18396,7 @@
       </c>
       <c r="F4" s="16" t="inlineStr">
         <is>
-          <t>vikram.singh@dzukku.com</t>
+          <t>vikram.singh@nourishbot.local</t>
         </is>
       </c>
       <c r="G4" s="16" t="inlineStr">
@@ -18463,7 +18463,7 @@
       </c>
       <c r="F5" s="16" t="inlineStr">
         <is>
-          <t>anjali.patel@dzukku.com</t>
+          <t>anjali.patel@nourishbot.local</t>
         </is>
       </c>
       <c r="G5" s="16" t="inlineStr">
@@ -18530,7 +18530,7 @@
       </c>
       <c r="F6" s="16" t="inlineStr">
         <is>
-          <t>sanjay.reddy@dzukku.com</t>
+          <t>sanjay.reddy@nourishbot.local</t>
         </is>
       </c>
       <c r="G6" s="16" t="inlineStr">
@@ -18597,7 +18597,7 @@
       </c>
       <c r="F7" s="16" t="inlineStr">
         <is>
-          <t>meera.iyer@dzukku.com</t>
+          <t>meera.iyer@nourishbot.local</t>
         </is>
       </c>
       <c r="G7" s="16" t="inlineStr">
@@ -18664,7 +18664,7 @@
       </c>
       <c r="F8" s="16" t="inlineStr">
         <is>
-          <t>arun.joshi@dzukku.com</t>
+          <t>arun.joshi@nourishbot.local</t>
         </is>
       </c>
       <c r="G8" s="16" t="inlineStr">
@@ -18731,7 +18731,7 @@
       </c>
       <c r="F9" s="16" t="inlineStr">
         <is>
-          <t>sunita.malhotra@dzukku.com</t>
+          <t>sunita.malhotra@nourishbot.local</t>
         </is>
       </c>
       <c r="G9" s="16" t="inlineStr">
@@ -18798,7 +18798,7 @@
       </c>
       <c r="F10" s="16" t="inlineStr">
         <is>
-          <t>rahul.nair@dzukku.com</t>
+          <t>rahul.nair@nourishbot.local</t>
         </is>
       </c>
       <c r="G10" s="16" t="inlineStr">
@@ -18865,7 +18865,7 @@
       </c>
       <c r="F11" s="16" t="inlineStr">
         <is>
-          <t>kavita.desai@dzukku.com</t>
+          <t>kavita.desai@nourishbot.local</t>
         </is>
       </c>
       <c r="G11" s="16" t="inlineStr">
@@ -18932,7 +18932,7 @@
       </c>
       <c r="F12" s="16" t="inlineStr">
         <is>
-          <t>manoj.tiwari@dzukku.com</t>
+          <t>manoj.tiwari@nourishbot.local</t>
         </is>
       </c>
       <c r="G12" s="16" t="inlineStr">
@@ -18999,7 +18999,7 @@
       </c>
       <c r="F13" s="16" t="inlineStr">
         <is>
-          <t>neha.gupta@dzukku.com</t>
+          <t>neha.gupta@nourishbot.local</t>
         </is>
       </c>
       <c r="G13" s="16" t="inlineStr">
@@ -19066,7 +19066,7 @@
       </c>
       <c r="F14" s="16" t="inlineStr">
         <is>
-          <t>amit.bose@dzukku.com</t>
+          <t>amit.bose@nourishbot.local</t>
         </is>
       </c>
       <c r="G14" s="16" t="inlineStr">
@@ -19133,7 +19133,7 @@
       </c>
       <c r="F15" s="16" t="inlineStr">
         <is>
-          <t>pooja.reddy@dzukku.com</t>
+          <t>pooja.reddy@nourishbot.local</t>
         </is>
       </c>
       <c r="G15" s="16" t="inlineStr">
@@ -19200,7 +19200,7 @@
       </c>
       <c r="F16" s="16" t="inlineStr">
         <is>
-          <t>rohit.kumar@dzukku.com</t>
+          <t>rohit.kumar@nourishbot.local</t>
         </is>
       </c>
       <c r="G16" s="16" t="inlineStr">
@@ -19267,7 +19267,7 @@
       </c>
       <c r="F17" s="16" t="inlineStr">
         <is>
-          <t>sonia.mehra@dzukku.com</t>
+          <t>sonia.mehra@nourishbot.local</t>
         </is>
       </c>
       <c r="G17" s="16" t="inlineStr">
@@ -19334,7 +19334,7 @@
       </c>
       <c r="F18" s="16" t="inlineStr">
         <is>
-          <t>vishal.nair@dzukku.com</t>
+          <t>vishal.nair@nourishbot.local</t>
         </is>
       </c>
       <c r="G18" s="16" t="inlineStr">
@@ -19401,7 +19401,7 @@
       </c>
       <c r="F19" s="16" t="inlineStr">
         <is>
-          <t>anita.sharma@dzukku.com</t>
+          <t>anita.sharma@nourishbot.local</t>
         </is>
       </c>
       <c r="G19" s="16" t="inlineStr">
@@ -19468,7 +19468,7 @@
       </c>
       <c r="F20" s="16" t="inlineStr">
         <is>
-          <t>deepak.singh@dzukku.com</t>
+          <t>deepak.singh@nourishbot.local</t>
         </is>
       </c>
       <c r="G20" s="16" t="inlineStr">
@@ -19535,7 +19535,7 @@
       </c>
       <c r="F21" s="16" t="inlineStr">
         <is>
-          <t>madhuri.patel@dzukku.com</t>
+          <t>madhuri.patel@nourishbot.local</t>
         </is>
       </c>
       <c r="G21" s="16" t="inlineStr">
@@ -37036,7 +37036,7 @@
       </c>
       <c r="D22" s="19" t="inlineStr">
         <is>
-          <t>Dzukku Restaurant</t>
+          <t>NourishBot Kitchen</t>
         </is>
       </c>
       <c r="F22" s="20" t="n">

</xml_diff>